<commit_message>
Update strategy docs for the new Tyumen tariffs
Describe the implemented rooms-based tariffs and the per-m2 follow-up,
and correct the earlier claim that engine time norms contradict the
site FAQ: they are visit durations for a two-person crew and match it.
Add the prior-price scenario under engine time norms, and label the
old seed tariffs as prior prices in the model and workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VgQJtx6Z9iSBdmfW52ZbzF
</commit_message>
<xml_diff>
--- a/strategy/model/cleanliness_finmodel.xlsx
+++ b/strategy/model/cleanliness_finmodel.xlsx
@@ -189,7 +189,7 @@
     <t xml:space="preserve">3. Сценарии отличаются только объёмами, оттоком и CAC (лист «Сценарии»); цены и затраты на заказ общие.</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Модель считается на РЕКОМЕНДУЕМОМ прайсе. Текущий прайс сайта (сиды) — для сравнения на листе «Юнит-экономика».</t>
+    <t xml:space="preserve">4. Модель считается на РЕКОМЕНДУЕМОМ прайсе. Прежний прайс сайта (сиды до обновления) — для сравнения на листе «Юнит-экономика».</t>
   </si>
   <si>
     <t xml:space="preserve">Цветовая легенда:</t>
@@ -642,7 +642,7 @@
     <t xml:space="preserve">Прямые затраты (ФОТ штатного клинера, химия, расходники), % выручки</t>
   </si>
   <si>
-    <t xml:space="preserve">Текущий прайс Тюмени из проекта (services/api/app/seed.py) — для сравнения</t>
+    <t xml:space="preserve">Прежний прайс Тюмени (seed.py на ревизии 0be802d) — для сравнения</t>
   </si>
   <si>
     <t xml:space="preserve">Типовой объект: комнат</t>
@@ -660,7 +660,7 @@
     <t xml:space="preserve">Поддерживающая: база</t>
   </si>
   <si>
-    <t xml:space="preserve">Сиды проекта, город tyumen</t>
+    <t xml:space="preserve">Сиды проекта до обновления, город tyumen</t>
   </si>
   <si>
     <t xml:space="preserve">Поддерживающая: за комнату</t>
@@ -1119,13 +1119,13 @@
     <t xml:space="preserve">Окупаемость CAC, мес</t>
   </si>
   <si>
-    <t xml:space="preserve">Текущий прайс сайта vs рекомендуемый (2-комн., 1 санузел)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Текущий: доля ФОТ как в модели</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Текущий: рыночная ставка клинера</t>
+    <t xml:space="preserve">Прежний прайс сайта vs рекомендуемый (2-комн., 1 санузел)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Прежний: доля ФОТ как в модели</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Прежний: рыночная ставка клинера</t>
   </si>
   <si>
     <t xml:space="preserve">Рекомендуемый прайс</t>

</xml_diff>